<commit_message>
ASC Mini-C3: ULN2003A driver, combo flow connector, assembly markings
- ULN2003A (LCSC C7512) drives the pump (ch 1+2) and the relay (ch 3);
  replaces 2 x AO3400A, 3 x B5819W and 4 resistors, as on FG1
- Flow input: one footprint takes a JST-XH (bench) or a 3.5 mm 3-pole
  screw terminal (FG1 field cable)
- Screw terminals now Phoenix PT-1,5 3.5 mm (KF350 type, library 3D);
  relay output is a pluggable MSTBVA 5.08 header like FG1's
- 1206 LEDs for hand soldering; ref + value labels on every part
  (R3 1K, U3 ULN2003 ...), "1" at IC pin 1, "+" at LED/diode anodes;
  back reads "Agri Sensors and Controls  Oct 2026"
- Re-routed, DRC clean (mains 5 mm), panel and fab regenerated
- Sourcing BOM: 1206 LED and ULN2003A LCSC numbers, CR2032 holder as an
  alternative to the tabbed cell; kit about Rs 967

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/ASC-StudentKit/hardware/MiniC3/sourcing/ASC-MiniC3-sourcing-BOM.xlsx
+++ b/products/ASC-StudentKit/hardware/MiniC3/sourcing/ASC-MiniC3-sourcing-BOM.xlsx
@@ -759,24 +759,24 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>MOSFET AO3400A</t>
+          <t>Schottky B5819W (flow level shift)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>SOT-23, LCSC C20917 (basic)</t>
+          <t>SOD-123, LCSC C8598 (basic)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Q1, Q2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -785,11 +785,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20917.html</t>
+          <t>https://www.lcsc.com/product-detail/C8598.html</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>7.9</v>
+        <v>2.5</v>
       </c>
       <c r="K9" s="4">
         <f>ROUND(G9*J9,0)</f>
@@ -802,7 +802,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 5</t>
+          <t>LCSC minimum 20</t>
         </is>
       </c>
     </row>
@@ -817,24 +817,24 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Schottky B5819W</t>
+          <t>Driver ULN2003A (pump on ch 1+2, relay on ch 3)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>SOD-123, LCSC C8598 (basic)</t>
+          <t>SOIC-16, TI ULN2003ADR, LCSC C7512</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>D1, D2, D6</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
@@ -843,11 +843,11 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C8598.html</t>
+          <t>https://www.lcsc.com/product-detail/C7512.html</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2.5</v>
+        <v>13.6</v>
       </c>
       <c r="K10" s="4">
         <f>ROUND(G10*J10,0)</f>
@@ -860,7 +860,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 20</t>
+          <t>LCSC minimum 5</t>
         </is>
       </c>
     </row>
@@ -875,12 +875,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 red (PUMP)</t>
+          <t>LED 1206 red (PUMP)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>LCSC C84256 (basic)</t>
+          <t>YONGYUTAI YLED1206RFT, LCSC C37635751</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -901,11 +901,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C84256.html</t>
+          <t>https://www.lcsc.com/product-detail/C37635751.html</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>1.19</v>
+        <v>1.77</v>
       </c>
       <c r="K11" s="4">
         <f>ROUND(G11*J11,0)</f>
@@ -933,12 +933,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 yellow (FLOW)</t>
+          <t>LED 1206 yellow (FLOW)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>LCSC C2296 (basic)</t>
+          <t>YLED1206Y, LCSC C30584802</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -959,11 +959,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2296.html</t>
+          <t>https://www.lcsc.com/product-detail/C30584802.html</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1.09</v>
+        <v>1.42</v>
       </c>
       <c r="K12" s="4">
         <f>ROUND(G12*J12,0)</f>
@@ -991,12 +991,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 green (STATUS)</t>
+          <t>LED 1206 green (STATUS)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>LCSC C2297 (basic)</t>
+          <t>YLED1206GFT, LCSC C37635752</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -1017,11 +1017,11 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2297.html</t>
+          <t>https://www.lcsc.com/product-detail/C37635752.html</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1.45</v>
+        <v>2.09</v>
       </c>
       <c r="K13" s="4">
         <f>ROUND(G13*J13,0)</f>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 50</t>
+          <t>LCSC minimum 20</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 blue (RELAY)</t>
+          <t>LED 1206 blue (RELAY)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>LCSC C84259</t>
+          <t>YLED1206B, LCSC C28310438</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1066,7 +1066,7 @@
         <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
@@ -1075,11 +1075,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C84259.html</t>
+          <t>https://www.lcsc.com/product-detail/C28310438.html</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2.36</v>
+        <v>1.39</v>
       </c>
       <c r="K14" s="4">
         <f>ROUND(G14*J14,0)</f>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 20</t>
+          <t>LCSC minimum 50</t>
         </is>
       </c>
     </row>
@@ -1107,21 +1107,21 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 100R</t>
+          <t>Resistor 0805 1k</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17408</t>
+          <t>LCSC C17513</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>R1, R10</t>
+          <t>R3, R4, R12</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>100</v>
@@ -1133,11 +1133,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17408.html</t>
+          <t>https://www.lcsc.com/product-detail/C17513.html</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.38</v>
+        <v>0.31</v>
       </c>
       <c r="K15" s="4">
         <f>ROUND(G15*J15,0)</f>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>LCSC reel-cut minimum 100</t>
+          <t>LCSC minimum 100</t>
         </is>
       </c>
     </row>
@@ -1165,21 +1165,21 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 100k</t>
+          <t>Resistor 0805 470R</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>LCSC C149504</t>
+          <t>LCSC C17710</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>R2, R11</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>100</v>
@@ -1191,11 +1191,11 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C149504.html</t>
+          <t>https://www.lcsc.com/product-detail/C17710.html</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.53</v>
+        <v>0.43</v>
       </c>
       <c r="K16" s="4">
         <f>ROUND(G16*J16,0)</f>
@@ -1223,21 +1223,21 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 1k</t>
+          <t>Resistor 0805 10k</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17513</t>
+          <t>LCSC C17414</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>R3, R4, R12</t>
+          <t>R6, R7</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>100</v>
@@ -1249,11 +1249,11 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17513.html</t>
+          <t>https://www.lcsc.com/product-detail/C17414.html</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="K17" s="4">
         <f>ROUND(G17*J17,0)</f>
@@ -1281,21 +1281,21 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 470R</t>
+          <t>Resistor 0805 4.7k</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17710</t>
+          <t>LCSC C17673</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R8, R9</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>100</v>
@@ -1307,11 +1307,11 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17710.html</t>
+          <t>https://www.lcsc.com/product-detail/C17673.html</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="K18" s="4">
         <f>ROUND(G18*J18,0)</f>
@@ -1339,24 +1339,24 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 10k</t>
+          <t>Capacitor 0805 100nF 50V</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17414</t>
+          <t>LCSC C49678</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>R6, R7</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
@@ -1365,11 +1365,11 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17414.html</t>
+          <t>https://www.lcsc.com/product-detail/C49678.html</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.3</v>
+        <v>1.68</v>
       </c>
       <c r="K19" s="4">
         <f>ROUND(G19*J19,0)</f>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 100</t>
+          <t>LCSC minimum 20</t>
         </is>
       </c>
     </row>
@@ -1397,24 +1397,24 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 4.7k</t>
+          <t>Capacitor 0805 10uF 25V (on the stick)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17673</t>
+          <t>LCSC C15850</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>R8, R9</t>
+          <t>C1 (stick)</t>
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
@@ -1423,11 +1423,11 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17673.html</t>
+          <t>https://www.lcsc.com/product-detail/C15850.html</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0.45</v>
+        <v>6.12</v>
       </c>
       <c r="K20" s="4">
         <f>ROUND(G20*J20,0)</f>
@@ -1440,65 +1440,65 @@
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 100</t>
+          <t>LCSC minimum 20</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>SMD (JLC assembly or LCSC)</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Capacitor 0805 100nF 50V</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>LCSC C49678</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="n">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>JLC SMT assembly share (if JLC assembles)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>setup + stencil + 3 extended-part fees (DS1307, AHT20, ULN2003A) over 80 sets</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>LCSC</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C49678.html</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="K21" s="4">
+      <c r="G21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>JLCPCB / WhyPCB</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>https://jlcpcb.com/smt-assembly</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3">
         <f>ROUND(G21*J21,0)</f>
         <v/>
       </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="M21" s="4" t="inlineStr">
-        <is>
-          <t>LCSC minimum 20</t>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Not for samples: hand-assemble (0805 parts; AHT20 with hot air)</t>
         </is>
       </c>
     </row>
@@ -1508,42 +1508,42 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SMD (JLC assembly or LCSC)</t>
+          <t>Through-hole (India)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Capacitor 0805 10uF 25V (on the stick)</t>
+          <t>ESP32-C3 Super Mini USB-C</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>LCSC C15850</t>
+          <t>plugs into the two 1x8 sockets</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>C1 (stick)</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>LCSC</t>
+          <t>Robosap</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15850.html</t>
+          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>6.12</v>
+        <v>238.36</v>
       </c>
       <c r="K22" s="4">
         <f>ROUND(G22*J22,0)</f>
@@ -1556,67 +1556,63 @@
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 20</t>
+          <t>2 + 1 spare</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>SMD (JLC assembly or LCSC)</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>JLC SMT assembly share (if JLC assembles)</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>setup + stencil + 2 extended-part fees over 80 sets</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>JLCPCB / WhyPCB</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>https://jlcpcb.com/smt-assembly</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="3">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Through-hole (India)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Female header 1x8 2.54 mm</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Super Mini socket, 8.5 mm tall</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Sharvi Electronics</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="K23" s="4">
         <f>ROUND(G23*J23,0)</f>
         <v/>
       </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>Not for samples: hand-assemble (0805 parts; AHT20 with hot air)</t>
-        </is>
-      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -1629,37 +1625,37 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>ESP32-C3 Super Mini USB-C</t>
+          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>plugs into the two 1x8 sockets</t>
+          <t>SPST-NO, sealed, VDE reinforced</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Robosap</t>
+          <t>techiesms</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
+          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>238.36</v>
+        <v>42</v>
       </c>
       <c r="K24" s="4">
         <f>ROUND(G24*J24,0)</f>
@@ -1672,7 +1668,7 @@
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>2 + 1 spare</t>
+          <t>Sold as a pack of 5 (Rs 210)</t>
         </is>
       </c>
     </row>
@@ -1687,37 +1683,37 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Female header 1x8 2.54 mm</t>
+          <t>CR2032 with 3 solder tabs, vertical</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Super Mini socket, 8.5 mm tall</t>
+          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>BT1</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Sharvi Electronics</t>
+          <t>Rajiv Electronics</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>10.72</v>
+        <v>29.5</v>
       </c>
       <c r="K25" s="4">
         <f>ROUND(G25*J25,0)</f>
@@ -1728,7 +1724,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>2 + 1 to measure the leg positions</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -1741,37 +1741,37 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
+          <t>ALTERNATIVE: CR2032 holder (vertical, 3 pins, Rajiv RBH-2) + loose CR2032 cell</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>SPST-NO, sealed, VDE reinforced</t>
+          <t>3-pin vertical holder; pin positions to be measured against the tabbed-cell pads</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>BT1 (alt)</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>techiesms</t>
+          <t>Rajiv Electronics</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-pcb-mount-vertical-battery-holder</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>42</v>
+        <v>11.8</v>
       </c>
       <c r="K26" s="4">
         <f>ROUND(G26*J26,0)</f>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>Sold as a pack of 5 (Rs 210)</t>
+          <t>Samples only, to measure the pins and judge quality</t>
         </is>
       </c>
     </row>
@@ -1799,17 +1799,17 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>CR2032 with 3 solder tabs, vertical</t>
+          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
+          <t>cylindrical</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>BT1</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
@@ -1820,16 +1820,16 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Rajiv Electronics</t>
+          <t>Magno Teknik</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
+          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>29.5</v>
+        <v>15</v>
       </c>
       <c r="K27" s="4">
         <f>ROUND(G27*J27,0)</f>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>2 + 1 to measure the leg positions</t>
+          <t>2 + 1 spare</t>
         </is>
       </c>
     </row>
@@ -1857,52 +1857,44 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
+          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>cylindrical</t>
+          <t>radial 5 x 11</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Magno Teknik</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="n">
-        <v>15</v>
       </c>
       <c r="K28" s="4">
         <f>ROUND(G28*J28,0)</f>
         <v/>
       </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
-        <is>
-          <t>2 + 1 spare</t>
-        </is>
-      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1915,33 +1907,33 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
+          <t>Screw terminal 3.5 mm 2P (PUMP)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>radial 5 x 11</t>
+          <t>KF350-2P / DG350 (Phoenix PT-1,5 footprint), horizontal</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="F29" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
+          <t>Local market (Lamington Rd / SP Road)</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K29" s="4">
         <f>ROUND(G29*J29,0)</f>
@@ -1952,117 +1944,117 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>Per kit: PUMP 2P + I2C 2P+2P + the 2P half of AUX = 4 x 2P</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Through-hole (India)</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Screw terminal 3.81 mm 2P (PUMP)</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>KF128-3.81 / KF2EDG, horizontal</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="n">
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Screw terminal 3.5 mm 4P (I2C)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>KF350 2P + 2P joined</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Local market (Lamington Rd / SP Road)</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>https://abra-electronics.com/interconnects/terminals-blocks-barrier/terminal-blocks/screw-terminal-blocks-stackable/tb-3-81mm-02-kf128-3-81mm-2-position-stackable-screw-terminal-block.html</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K30" s="4">
+      <c r="G30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3">
         <f>ROUND(G30*J30,0)</f>
         <v/>
       </c>
-      <c r="L30" s="7" t="inlineStr">
+      <c r="L30" s="6" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
-        <is>
-          <t>Per kit: 2P (PUMP) + 2P+2P (I2C) + 2P of the 5P = 4 x 2P</t>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Made from 2 x 2P (counted in the 2P line)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Through-hole (India)</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Screw terminal 3.81 mm 4P (I2C)</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>KF128-3.81 2P + 2P stacked</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>J5</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="n">
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Screw terminal 3.5 mm 5P (AUX)</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>KF350 2P + 3P joined</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="G31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Local market</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="3">
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K31" s="4">
         <f>ROUND(G31*J31,0)</f>
         <v/>
       </c>
-      <c r="L31" s="6" t="inlineStr">
+      <c r="L31" s="7" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>Made from 2 x 2P (counted in the 2P line)</t>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>3P half of the 5P (the 2P half is in the 2P line)</t>
         </is>
       </c>
     </row>
@@ -2077,21 +2069,21 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.81 mm 5P (AUX)</t>
+          <t>Screw terminal 3.5 mm 3P (FLOW, field builds)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>KF128-3.81 2P + 3P stacked</t>
+          <t>KF350-3P; fits the same holes as the JST-XH</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J4 (alt)</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>2</v>
@@ -2103,7 +2095,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr"/>
       <c r="J32" s="4" t="n">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="K32" s="4">
         <f>ROUND(G32*J32,0)</f>
@@ -2116,7 +2108,7 @@
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>3P part; 2P + 3P stacked = 5P</t>
+          <t>For testing the field (terminal) build of the flow input</t>
         </is>
       </c>
     </row>
@@ -2131,12 +2123,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 5.08 mm 2P (RELAY 230 V)</t>
+          <t>Pluggable header 5.08 mm 2P, vertical, + plug (RELAY 230 V)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>KF301-2P</t>
+          <t>MSTBVA 2,5/2-G-5,08 type (2EDG-V 5.08) with 2EDGK plug</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2152,7 +2144,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>ElectronicsComp</t>
+          <t>Local market</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -2161,18 +2153,22 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>22.4</v>
+        <v>15</v>
       </c>
       <c r="K33" s="4">
         <f>ROUND(G33*J33,0)</f>
         <v/>
       </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="M33" s="4" t="inlineStr"/>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Header + plug pairs</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -2185,12 +2181,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>JST-XH 3-pin male header, straight 2.5 mm</t>
+          <t>JST-XH 3-pin male header, straight 2.5 mm (FLOW, student builds)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>B3B-XH-A type</t>
+          <t>B3B-XH-A type; shares the footprint with the 3.5 mm terminal</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2764,15 +2760,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3089,21 +3083,21 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MOSFET AO3400A</t>
+          <t>Schottky B5819W (flow level shift)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>SOT-23, LCSC C20917 (basic)</t>
+          <t>SOD-123, LCSC C8598 (basic)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Q1, Q2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4">
         <f>CEILING(F8*80,1)</f>
@@ -3116,11 +3110,11 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C20917.html</t>
+          <t>https://www.lcsc.com/product-detail/C8598.html</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6.4</v>
+        <v>1.9</v>
       </c>
       <c r="K8" s="4">
         <f>ROUND(F8*J8,2)</f>
@@ -3148,21 +3142,21 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Schottky B5819W</t>
+          <t>Driver ULN2003A (pump on ch 1+2, relay on ch 3)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>SOD-123, LCSC C8598 (basic)</t>
+          <t>SOIC-16, TI ULN2003ADR, LCSC C7512</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>D1, D2, D6</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4">
         <f>CEILING(F9*80,1)</f>
@@ -3175,11 +3169,11 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C8598.html</t>
+          <t>https://www.lcsc.com/product-detail/C7512.html</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>1.9</v>
+        <v>10.4</v>
       </c>
       <c r="K9" s="4">
         <f>ROUND(F9*J9,2)</f>
@@ -3194,7 +3188,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Replaces 2 x AO3400A, 3 x B5819W and 4 resistors; same driver as FG1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -3207,12 +3205,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 red (PUMP)</t>
+          <t>LED 1206 red (PUMP)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>LCSC C84256 (basic)</t>
+          <t>YONGYUTAI YLED1206RFT, LCSC C37635751</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -3234,11 +3232,11 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C84256.html</t>
+          <t>https://www.lcsc.com/product-detail/C37635751.html</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="K10" s="4">
         <f>ROUND(F10*J10,2)</f>
@@ -3253,7 +3251,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>1206 for hand soldering, as on WPC</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -3266,12 +3268,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 yellow (FLOW)</t>
+          <t>LED 1206 yellow (FLOW)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>LCSC C2296 (basic)</t>
+          <t>YLED1206Y, LCSC C30584802</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -3293,11 +3295,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2296.html</t>
+          <t>https://www.lcsc.com/product-detail/C30584802.html</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="K11" s="4">
         <f>ROUND(F11*J11,2)</f>
@@ -3325,12 +3327,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 green (STATUS)</t>
+          <t>LED 1206 green (STATUS)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>LCSC C2297 (basic)</t>
+          <t>YLED1206GFT, LCSC C37635752</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -3352,11 +3354,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C2297.html</t>
+          <t>https://www.lcsc.com/product-detail/C37635752.html</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="K12" s="4">
         <f>ROUND(F12*J12,2)</f>
@@ -3384,12 +3386,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>LED 0805 blue (RELAY)</t>
+          <t>LED 1206 blue (RELAY)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>LCSC C84259</t>
+          <t>YLED1206B, LCSC C28310438</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -3411,11 +3413,11 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C84259.html</t>
+          <t>https://www.lcsc.com/product-detail/C28310438.html</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="K13" s="4">
         <f>ROUND(F13*J13,2)</f>
@@ -3430,7 +3432,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Low stock at LCSC (450 on 2026-10-11)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -3443,21 +3449,21 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 100R</t>
+          <t>Resistor 0805 1k</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17408</t>
+          <t>LCSC C17513</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>R1, R10</t>
+          <t>R3, R4, R12</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="4">
         <f>CEILING(F14*80,1)</f>
@@ -3470,11 +3476,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17408.html</t>
+          <t>https://www.lcsc.com/product-detail/C17513.html</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.38</v>
+        <v>0.31</v>
       </c>
       <c r="K14" s="4">
         <f>ROUND(F14*J14,2)</f>
@@ -3502,21 +3508,21 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 100k</t>
+          <t>Resistor 0805 470R</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>LCSC C149504</t>
+          <t>LCSC C17710</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>R2, R11</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" s="4">
         <f>CEILING(F15*80,1)</f>
@@ -3529,11 +3535,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C149504.html</t>
+          <t>https://www.lcsc.com/product-detail/C17710.html</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.53</v>
+        <v>0.43</v>
       </c>
       <c r="K15" s="4">
         <f>ROUND(F15*J15,2)</f>
@@ -3561,21 +3567,21 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 1k</t>
+          <t>Resistor 0805 10k</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17513</t>
+          <t>LCSC C17414</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>R3, R4, R12</t>
+          <t>R6, R7</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16" s="4">
         <f>CEILING(F16*80,1)</f>
@@ -3588,11 +3594,11 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17513.html</t>
+          <t>https://www.lcsc.com/product-detail/C17414.html</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="K16" s="4">
         <f>ROUND(F16*J16,2)</f>
@@ -3620,21 +3626,21 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 470R</t>
+          <t>Resistor 0805 4.7k</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17710</t>
+          <t>LCSC C17673</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R8, R9</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="4">
         <f>CEILING(F17*80,1)</f>
@@ -3647,11 +3653,11 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17710.html</t>
+          <t>https://www.lcsc.com/product-detail/C17673.html</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="K17" s="4">
         <f>ROUND(F17*J17,2)</f>
@@ -3679,21 +3685,21 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 10k</t>
+          <t>Capacitor 0805 100nF 50V</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17414</t>
+          <t>LCSC C49678</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>R6, R7</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G18" s="4">
         <f>CEILING(F18*80,1)</f>
@@ -3706,11 +3712,11 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17414.html</t>
+          <t>https://www.lcsc.com/product-detail/C49678.html</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="K18" s="4">
         <f>ROUND(F18*J18,2)</f>
@@ -3738,21 +3744,21 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 4.7k</t>
+          <t>Capacitor 0805 10uF 25V (on the stick)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17673</t>
+          <t>LCSC C15850</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>R8, R9</t>
+          <t>C1 (stick)</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="4">
         <f>CEILING(F19*80,1)</f>
@@ -3765,11 +3771,11 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17673.html</t>
+          <t>https://www.lcsc.com/product-detail/C15850.html</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.45</v>
+        <v>4.5</v>
       </c>
       <c r="K19" s="4">
         <f>ROUND(F19*J19,2)</f>
@@ -3797,17 +3803,17 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Capacitor 0805 100nF 50V</t>
+          <t>JLC SMT assembly share (if JLC assembles)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>LCSC C49678</t>
+          <t>setup + stencil + 3 extended-part fees (DS1307, AHT20, ULN2003A) over 80 sets</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F20" s="4" t="n">
@@ -3819,16 +3825,16 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>LCSC</t>
+          <t>JLCPCB / WhyPCB</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49678.html</t>
+          <t>https://jlcpcb.com/smt-assembly</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>1.2</v>
+        <v>25</v>
       </c>
       <c r="K20" s="4">
         <f>ROUND(F20*J20,2)</f>
@@ -3838,12 +3844,16 @@
         <f>ROUND(F20*80*J20,0)</f>
         <v/>
       </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>Skip if hand-assembled; the AHT20 still needs reflow or hot air</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -3851,22 +3861,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SMD (JLC assembly or LCSC)</t>
+          <t>Through-hole (India)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Capacitor 0805 10uF 25V (on the stick)</t>
+          <t>ESP32-C3 Super Mini USB-C</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>LCSC C15850</t>
+          <t>plugs into the two 1x8 sockets</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>C1 (stick)</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="F21" s="4" t="n">
@@ -3878,16 +3888,16 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>LCSC</t>
+          <t>Robosap</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15850.html</t>
+          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>4.5</v>
+        <v>238.36</v>
       </c>
       <c r="K21" s="4">
         <f>ROUND(F21*J21,2)</f>
@@ -3902,7 +3912,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Rs 202 + GST; check the pin order against the 1:1 print</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -3910,26 +3924,26 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SMD (JLC assembly or LCSC)</t>
+          <t>Through-hole (India)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>JLC SMT assembly share (if JLC assembles)</t>
+          <t>Female header 1x8 2.54 mm</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>setup + stencil + 2 extended-part fees over 80 sets</t>
+          <t>Super Mini socket, 8.5 mm tall</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="4">
         <f>CEILING(F22*80,1)</f>
@@ -3937,16 +3951,16 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>JLCPCB / WhyPCB</t>
+          <t>Sharvi Electronics</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>https://jlcpcb.com/smt-assembly</t>
+          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>25</v>
+        <v>10.72</v>
       </c>
       <c r="K22" s="4">
         <f>ROUND(F22*J22,2)</f>
@@ -3956,16 +3970,12 @@
         <f>ROUND(F22*80*J22,0)</f>
         <v/>
       </c>
-      <c r="M22" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>Skip if hand-assembled; the AHT20 still needs reflow or hot air</t>
-        </is>
-      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -3978,17 +3988,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>ESP32-C3 Super Mini USB-C</t>
+          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>plugs into the two 1x8 sockets</t>
+          <t>SPST-NO, sealed, VDE reinforced</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="F23" s="4" t="n">
@@ -4000,16 +4010,16 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Robosap</t>
+          <t>techiesms</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
+          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>238.36</v>
+        <v>42</v>
       </c>
       <c r="K23" s="4">
         <f>ROUND(F23*J23,2)</f>
@@ -4026,7 +4036,7 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Rs 202 + GST; check the pin order against the 1:1 print</t>
+          <t>Rs 210 for a pack of 5</t>
         </is>
       </c>
     </row>
@@ -4041,21 +4051,21 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Female header 1x8 2.54 mm</t>
+          <t>CR2032 with 3 solder tabs, vertical</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Super Mini socket, 8.5 mm tall</t>
+          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>BT1</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" s="4">
         <f>CEILING(F24*80,1)</f>
@@ -4063,16 +4073,16 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Sharvi Electronics</t>
+          <t>Rajiv Electronics</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>10.72</v>
+        <v>29.5</v>
       </c>
       <c r="K24" s="4">
         <f>ROUND(F24*J24,2)</f>
@@ -4087,7 +4097,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>Measure the - leg offset on the first lot (footprint assumes 4.0 mm)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -4100,21 +4114,21 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
+          <t>ALTERNATIVE: CR2032 holder (vertical, 3 pins, Rajiv RBH-2) + loose CR2032 cell</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>SPST-NO, sealed, VDE reinforced</t>
+          <t>3-pin vertical holder; pin positions to be measured against the tabbed-cell pads</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>BT1 (alt)</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25" s="4">
         <f>CEILING(F25*80,1)</f>
@@ -4122,16 +4136,16 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>techiesms</t>
+          <t>Rajiv Electronics</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-pcb-mount-vertical-battery-holder</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>42</v>
+        <v>11.8</v>
       </c>
       <c r="K25" s="4">
         <f>ROUND(F25*J25,2)</f>
@@ -4148,7 +4162,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>Rs 210 for a pack of 5</t>
+          <t>Rs 11.80 + a loose CR2032 (about Rs 20). Replaceable cell. Measure a sample: if its 3 pins match the tabbed-cell pads it drops in, otherwise we add its pads</t>
         </is>
       </c>
     </row>
@@ -4163,17 +4177,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>CR2032 with 3 solder tabs, vertical</t>
+          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
+          <t>cylindrical</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>BT1</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
@@ -4185,16 +4199,16 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Rajiv Electronics</t>
+          <t>Magno Teknik</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
+          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>29.5</v>
+        <v>14</v>
       </c>
       <c r="K26" s="4">
         <f>ROUND(F26*J26,2)</f>
@@ -4211,7 +4225,7 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Measure the - leg offset on the first lot (footprint assumes 4.0 mm)</t>
+          <t>Rs 14 at 100+; local market about Rs 4-8</t>
         </is>
       </c>
     </row>
@@ -4226,17 +4240,17 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
+          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>cylindrical</t>
+          <t>radial 5 x 11</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
@@ -4248,16 +4262,12 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Magno Teknik</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
       <c r="J27" s="4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K27" s="4">
         <f>ROUND(F27*J27,2)</f>
@@ -4267,16 +4277,12 @@
         <f>ROUND(F27*80*J27,0)</f>
         <v/>
       </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>Rs 14 at 100+; local market about Rs 4-8</t>
-        </is>
-      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -4289,17 +4295,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
+          <t>Screw terminal 3.5 mm 2P (PUMP)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>radial 5 x 11</t>
+          <t>KF350-2P / DG350 (Phoenix PT-1,5 footprint), horizontal</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
@@ -4311,12 +4317,12 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
+          <t>Local market (Lamington Rd / SP Road)</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr"/>
       <c r="J28" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K28" s="4">
         <f>ROUND(F28*J28,2)</f>
@@ -4331,7 +4337,11 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>3.5 mm pitch blocks interlock: buy 2P and 3P and join them</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -4344,17 +4354,17 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.81 mm 2P (PUMP)</t>
+          <t>Screw terminal 3.5 mm 4P (I2C)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>KF128-3.81 / KF2EDG, horizontal</t>
+          <t>KF350 2P + 2P joined</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="F29" s="4" t="n">
@@ -4366,16 +4376,12 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Local market (Lamington Rd / SP Road)</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>https://abra-electronics.com/interconnects/terminals-blocks-barrier/terminal-blocks/screw-terminal-blocks-stackable/tb-3-81mm-02-kf128-3-81mm-2-position-stackable-screw-terminal-block.html</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K29" s="4">
         <f>ROUND(F29*J29,2)</f>
@@ -4392,7 +4398,7 @@
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>KF128 is stackable: buy 2P and 3P and join them for 4P and 5P. Link is a reference listing only</t>
+          <t>Wire entry faces the board edge</t>
         </is>
       </c>
     </row>
@@ -4407,17 +4413,17 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.81 mm 4P (I2C)</t>
+          <t>Screw terminal 3.5 mm 5P (AUX)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>KF128-3.81 2P + 2P stacked</t>
+          <t>KF350 2P + 3P joined</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="F30" s="4" t="n">
@@ -4449,11 +4455,7 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>Wire entry must face the board edge</t>
-        </is>
-      </c>
+      <c r="N30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -4466,21 +4468,21 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.81 mm 5P (AUX)</t>
+          <t>Screw terminal 3.5 mm 3P (FLOW, field builds)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>KF128-3.81 2P + 3P stacked</t>
+          <t>KF350-3P; fits the same holes as the JST-XH</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J4 (alt)</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" s="4">
         <f>CEILING(F31*80,1)</f>
@@ -4493,7 +4495,7 @@
       </c>
       <c r="I31" s="4" t="inlineStr"/>
       <c r="J31" s="4" t="n">
-        <v>12.5</v>
+        <v>6</v>
       </c>
       <c r="K31" s="4">
         <f>ROUND(F31*J31,2)</f>
@@ -4508,7 +4510,11 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>FG1 / long cable: fit this instead of the JST-XH header</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -4521,12 +4527,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 5.08 mm 2P (RELAY 230 V)</t>
+          <t>Pluggable header 5.08 mm 2P, vertical, + plug (RELAY 230 V)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>KF301-2P</t>
+          <t>MSTBVA 2,5/2-G-5,08 type (2EDG-V 5.08) with 2EDGK plug</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -4543,7 +4549,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>ElectronicsComp</t>
+          <t>Local market</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -4552,7 +4558,7 @@
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>22.4</v>
+        <v>15</v>
       </c>
       <c r="K32" s="4">
         <f>ROUND(F32*J32,2)</f>
@@ -4562,14 +4568,14 @@
         <f>ROUND(F32*80*J32,0)</f>
         <v/>
       </c>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Rs 19 + GST; Sharvi lists Rs 9.25 + tax</t>
+          <t>Same pluggable family as FG1's relay connector; buy header and plug as a pair (link: similar plug-in block)</t>
         </is>
       </c>
     </row>
@@ -4584,12 +4590,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>JST-XH 3-pin male header, straight 2.5 mm</t>
+          <t>JST-XH 3-pin male header, straight 2.5 mm (FLOW, student builds)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>B3B-XH-A type</t>
+          <t>B3B-XH-A type; shares the footprint with the 3.5 mm terminal</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -5272,15 +5278,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ASC Mini-C3: LED colours, relay header turned, date line
- LEDs: PUMP and RLY yellow (C30584802), STATUS red (C37635751),
  FLOW yellow-green (C28310441, ~2 V: it runs from 3.3 V into the
  sensor output); the Super Mini's blue LED on GPIO8 is the WiFi LED
- Relay MSTBVA header turned 180 so the curved side faces inward, as on
  FG1; pins re-mapped (1 COM, 2 NO), mains tracks re-drawn, 5.00 mm
- Back silkscreen: "Oct 2026" on its own line
- Re-routed, DRC clean; panel, fab, BOM/CPL and sourcing regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/ASC-StudentKit/hardware/MiniC3/sourcing/ASC-MiniC3-sourcing-BOM.xlsx
+++ b/products/ASC-StudentKit/hardware/MiniC3/sourcing/ASC-MiniC3-sourcing-BOM.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -875,21 +875,21 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 red (PUMP)</t>
+          <t>LED 1206 yellow (PUMP, RELAY)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>YONGYUTAI YLED1206RFT, LCSC C37635751</t>
+          <t>YONGYUTAI YLED1206Y, LCSC C30584802</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D3, D7</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>50</v>
@@ -901,11 +901,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C37635751.html</t>
+          <t>https://www.lcsc.com/product-detail/C30584802.html</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>1.77</v>
+        <v>1.42</v>
       </c>
       <c r="K11" s="4">
         <f>ROUND(G11*J11,0)</f>
@@ -933,17 +933,17 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 yellow (FLOW)</t>
+          <t>LED 1206 red (STATUS)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>YLED1206Y, LCSC C30584802</t>
+          <t>YLED1206RFT, LCSC C37635751</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
@@ -959,11 +959,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C30584802.html</t>
+          <t>https://www.lcsc.com/product-detail/C37635751.html</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1.42</v>
+        <v>1.77</v>
       </c>
       <c r="K12" s="4">
         <f>ROUND(G12*J12,0)</f>
@@ -991,24 +991,24 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 green (STATUS)</t>
+          <t>LED 1206 yellow-green (FLOW)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>YLED1206GFT, LCSC C37635752</t>
+          <t>YLED1206YG 576 nm, LCSC C28310441</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -1017,11 +1017,11 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C37635752.html</t>
+          <t>https://www.lcsc.com/product-detail/C28310441.html</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>2.09</v>
+        <v>1.42</v>
       </c>
       <c r="K13" s="4">
         <f>ROUND(G13*J13,0)</f>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 20</t>
+          <t>LCSC minimum 50</t>
         </is>
       </c>
     </row>
@@ -1049,24 +1049,24 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 blue (RELAY)</t>
+          <t>Resistor 0805 1k</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>YLED1206B, LCSC C28310438</t>
+          <t>LCSC C17513</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>R3, R4, R12</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
@@ -1075,11 +1075,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C28310438.html</t>
+          <t>https://www.lcsc.com/product-detail/C17513.html</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1.39</v>
+        <v>0.31</v>
       </c>
       <c r="K14" s="4">
         <f>ROUND(G14*J14,0)</f>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 50</t>
+          <t>LCSC minimum 100</t>
         </is>
       </c>
     </row>
@@ -1107,21 +1107,21 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 1k</t>
+          <t>Resistor 0805 470R</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17513</t>
+          <t>LCSC C17710</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>R3, R4, R12</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>100</v>
@@ -1133,11 +1133,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17513.html</t>
+          <t>https://www.lcsc.com/product-detail/C17710.html</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.31</v>
+        <v>0.43</v>
       </c>
       <c r="K15" s="4">
         <f>ROUND(G15*J15,0)</f>
@@ -1165,21 +1165,21 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 470R</t>
+          <t>Resistor 0805 10k</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17710</t>
+          <t>LCSC C17414</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R6, R7</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>100</v>
@@ -1191,11 +1191,11 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17710.html</t>
+          <t>https://www.lcsc.com/product-detail/C17414.html</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.43</v>
+        <v>0.3</v>
       </c>
       <c r="K16" s="4">
         <f>ROUND(G16*J16,0)</f>
@@ -1223,17 +1223,17 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 10k</t>
+          <t>Resistor 0805 4.7k</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17414</t>
+          <t>LCSC C17673</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>R6, R7</t>
+          <t>R8, R9</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
@@ -1249,11 +1249,11 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17414.html</t>
+          <t>https://www.lcsc.com/product-detail/C17673.html</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K17" s="4">
         <f>ROUND(G17*J17,0)</f>
@@ -1281,24 +1281,24 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 4.7k</t>
+          <t>Capacitor 0805 100nF 50V</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17673</t>
+          <t>LCSC C49678</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>R8, R9</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
@@ -1307,11 +1307,11 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17673.html</t>
+          <t>https://www.lcsc.com/product-detail/C49678.html</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>0.45</v>
+        <v>1.68</v>
       </c>
       <c r="K18" s="4">
         <f>ROUND(G18*J18,0)</f>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>LCSC minimum 100</t>
+          <t>LCSC minimum 20</t>
         </is>
       </c>
     </row>
@@ -1339,17 +1339,17 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Capacitor 0805 100nF 50V</t>
+          <t>Capacitor 0805 10uF 25V (on the stick)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>LCSC C49678</t>
+          <t>LCSC C15850</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C1 (stick)</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">
@@ -1365,11 +1365,11 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49678.html</t>
+          <t>https://www.lcsc.com/product-detail/C15850.html</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>1.68</v>
+        <v>6.12</v>
       </c>
       <c r="K19" s="4">
         <f>ROUND(G19*J19,0)</f>
@@ -1387,118 +1387,118 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>SMD (JLC assembly or LCSC)</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Capacitor 0805 10uF 25V (on the stick)</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>LCSC C15850</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>C1 (stick)</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="n">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>JLC SMT assembly share (if JLC assembles)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>setup + stencil + 3 extended-part fees (DS1307, AHT20, ULN2003A) over 80 sets</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>LCSC</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>https://www.lcsc.com/product-detail/C15850.html</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="K20" s="4">
+      <c r="G20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>JLCPCB / WhyPCB</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>https://jlcpcb.com/smt-assembly</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3">
         <f>ROUND(G20*J20,0)</f>
         <v/>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Not for samples: hand-assemble (0805 parts; AHT20 with hot air)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Through-hole (India)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>ESP32-C3 Super Mini USB-C</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>plugs into the two 1x8 sockets</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Robosap</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>238.36</v>
+      </c>
+      <c r="K21" s="4">
+        <f>ROUND(G21*J21,0)</f>
+        <v/>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>quoted</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>LCSC minimum 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>SMD (JLC assembly or LCSC)</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>JLC SMT assembly share (if JLC assembles)</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>setup + stencil + 3 extended-part fees (DS1307, AHT20, ULN2003A) over 80 sets</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>JLCPCB / WhyPCB</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>https://jlcpcb.com/smt-assembly</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="3">
-        <f>ROUND(G21*J21,0)</f>
-        <v/>
-      </c>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Not for samples: hand-assemble (0805 parts; AHT20 with hot air)</t>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>2 + 1 spare</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>ESP32-C3 Super Mini USB-C</t>
+          <t>Female header 1x8 2.54 mm</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>plugs into the two 1x8 sockets</t>
+          <t>Super Mini socket, 8.5 mm tall</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1527,23 +1527,23 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Robosap</t>
+          <t>Sharvi Electronics</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
+          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>238.36</v>
+        <v>10.72</v>
       </c>
       <c r="K22" s="4">
         <f>ROUND(G22*J22,0)</f>
@@ -1554,11 +1554,7 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>2 + 1 spare</t>
-        </is>
-      </c>
+      <c r="M22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1571,37 +1567,37 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Female header 1x8 2.54 mm</t>
+          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Super Mini socket, 8.5 mm tall</t>
+          <t>SPST-NO, sealed, VDE reinforced</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Sharvi Electronics</t>
+          <t>techiesms</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
+          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>10.72</v>
+        <v>42</v>
       </c>
       <c r="K23" s="4">
         <f>ROUND(G23*J23,0)</f>
@@ -1612,7 +1608,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>Sold as a pack of 5 (Rs 210)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -1625,37 +1625,37 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
+          <t>CR2032 with 3 solder tabs, vertical</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>SPST-NO, sealed, VDE reinforced</t>
+          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>BT1</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>techiesms</t>
+          <t>Rajiv Electronics</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>42</v>
+        <v>29.5</v>
       </c>
       <c r="K24" s="4">
         <f>ROUND(G24*J24,0)</f>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>Sold as a pack of 5 (Rs 210)</t>
+          <t>2 + 1 to measure the leg positions</t>
         </is>
       </c>
     </row>
@@ -1683,25 +1683,25 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>CR2032 with 3 solder tabs, vertical</t>
+          <t>ALTERNATIVE: CR2032 holder (vertical, 3 pins, Rajiv RBH-2) + loose CR2032 cell</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
+          <t>3-pin vertical holder; pin positions to be measured against the tabbed-cell pads</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>BT1</t>
+          <t>BT1 (alt)</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Rajiv Electronics</t>
@@ -1709,11 +1709,11 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-pcb-mount-vertical-battery-holder</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>29.5</v>
+        <v>11.8</v>
       </c>
       <c r="K25" s="4">
         <f>ROUND(G25*J25,0)</f>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>2 + 1 to measure the leg positions</t>
+          <t>Samples only, to measure the pins and judge quality</t>
         </is>
       </c>
     </row>
@@ -1741,37 +1741,37 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>ALTERNATIVE: CR2032 holder (vertical, 3 pins, Rajiv RBH-2) + loose CR2032 cell</t>
+          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>3-pin vertical holder; pin positions to be measured against the tabbed-cell pads</t>
+          <t>cylindrical</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>BT1 (alt)</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Rajiv Electronics</t>
+          <t>Magno Teknik</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>https://rajivelectronics.com/product/cr2032-3v-pcb-mount-vertical-battery-holder</t>
+          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>11.8</v>
+        <v>15</v>
       </c>
       <c r="K26" s="4">
         <f>ROUND(G26*J26,0)</f>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>Samples only, to measure the pins and judge quality</t>
+          <t>2 + 1 spare</t>
         </is>
       </c>
     </row>
@@ -1799,52 +1799,44 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
+          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>cylindrical</t>
+          <t>radial 5 x 11</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>Magno Teknik</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="n">
-        <v>15</v>
       </c>
       <c r="K27" s="4">
         <f>ROUND(G27*J27,0)</f>
         <v/>
       </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>2 + 1 spare</t>
-        </is>
-      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -1857,33 +1849,33 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
+          <t>Screw terminal 3.5 mm 2P (PUMP)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>radial 5 x 11</t>
+          <t>KF350-2P / DG350 (Phoenix PT-1,5 footprint), horizontal</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
+          <t>Local market (Lamington Rd / SP Road)</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr"/>
       <c r="J28" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K28" s="4">
         <f>ROUND(G28*J28,0)</f>
@@ -1894,113 +1886,117 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>Per kit: PUMP 2P + I2C 2P+2P + the 2P half of AUX = 4 x 2P</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Through-hole (India)</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Screw terminal 3.5 mm 2P (PUMP)</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>KF350-2P / DG350 (Phoenix PT-1,5 footprint), horizontal</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n">
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Screw terminal 3.5 mm 4P (I2C)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>KF350 2P + 2P joined</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>Local market (Lamington Rd / SP Road)</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K29" s="4">
+      <c r="G29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="3">
         <f>ROUND(G29*J29,0)</f>
         <v/>
       </c>
-      <c r="L29" s="7" t="inlineStr">
+      <c r="L29" s="6" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr">
-        <is>
-          <t>Per kit: PUMP 2P + I2C 2P+2P + the 2P half of AUX = 4 x 2P</t>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Made from 2 x 2P (counted in the 2P line)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Through-hole (India)</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Screw terminal 3.5 mm 4P (I2C)</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>KF350 2P + 2P joined</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>J5</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="n">
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Screw terminal 3.5 mm 5P (AUX)</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>KF350 2P + 3P joined</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="G30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Local market</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="3">
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K30" s="4">
         <f>ROUND(G30*J30,0)</f>
         <v/>
       </c>
-      <c r="L30" s="6" t="inlineStr">
+      <c r="L30" s="7" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>Made from 2 x 2P (counted in the 2P line)</t>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>3P half of the 5P (the 2P half is in the 2P line)</t>
         </is>
       </c>
     </row>
@@ -2015,21 +2011,21 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.5 mm 5P (AUX)</t>
+          <t>Screw terminal 3.5 mm 3P (FLOW, field builds)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>KF350 2P + 3P joined</t>
+          <t>KF350-3P; fits the same holes as the JST-XH</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J4 (alt)</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>2</v>
@@ -2054,7 +2050,7 @@
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>3P half of the 5P (the 2P half is in the 2P line)</t>
+          <t>For testing the field (terminal) build of the flow input</t>
         </is>
       </c>
     </row>
@@ -2069,21 +2065,21 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.5 mm 3P (FLOW, field builds)</t>
+          <t>Pluggable header 5.08 mm 2P, vertical, + plug (RELAY 230 V)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>KF350-3P; fits the same holes as the JST-XH</t>
+          <t>MSTBVA 2,5/2-G-5,08 type (2EDG-V 5.08) with 2EDGK plug</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>J4 (alt)</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>2</v>
@@ -2093,9 +2089,13 @@
           <t>Local market</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr"/>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.electronicscomp.com/kf301-2-pin-5.08mm-pitch-plug-in-screw-terminal-block-connector</t>
+        </is>
+      </c>
       <c r="J32" s="4" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K32" s="4">
         <f>ROUND(G32*J32,0)</f>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>For testing the field (terminal) build of the flow input</t>
+          <t>Header + plug pairs</t>
         </is>
       </c>
     </row>
@@ -2123,50 +2123,50 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Pluggable header 5.08 mm 2P, vertical, + plug (RELAY 230 V)</t>
+          <t>JST-XH 3-pin male header, straight 2.5 mm (FLOW, student builds)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>MSTBVA 2,5/2-G-5,08 type (2EDG-V 5.08) with 2EDGK plug</t>
+          <t>B3B-XH-A type; shares the footprint with the 3.5 mm terminal</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="F33" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
+          <t>DNA Technology</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>https://www.electronicscomp.com/kf301-2-pin-5.08mm-pitch-plug-in-screw-terminal-block-connector</t>
+          <t>https://www.dnatechindia.com/3-pin-2-50mm-jst-xh-straight-male-connector-buy-in-india.html</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>15</v>
+        <v>4.56</v>
       </c>
       <c r="K33" s="4">
         <f>ROUND(G33*J33,0)</f>
         <v/>
       </c>
-      <c r="L33" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr">
         <is>
-          <t>Header + plug pairs</t>
+          <t>2 + 1 spare</t>
         </is>
       </c>
     </row>
@@ -2176,42 +2176,42 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Through-hole (India)</t>
+          <t>Kit items</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>JST-XH 3-pin male header, straight 2.5 mm (FLOW, student builds)</t>
+          <t>Flow sensor YF-S401 0.3-6 L/min</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>B3B-XH-A type; shares the footprint with the 3.5 mm terminal</t>
+          <t>5880 pulses per litre, JST-XH lead</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>DNA Technology</t>
+          <t>AM Electronics</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>https://www.dnatechindia.com/3-pin-2-50mm-jst-xh-straight-male-connector-buy-in-india.html</t>
+          <t>https://amelectronics.in/product/water-flow-sensor-yf-s401-flowmeter-0-3-6l-min-3-5mm-white/</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>4.56</v>
+        <v>230</v>
       </c>
       <c r="K34" s="4">
         <f>ROUND(G34*J34,0)</f>
@@ -2222,11 +2222,7 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M34" s="4" t="inlineStr">
-        <is>
-          <t>2 + 1 spare</t>
-        </is>
-      </c>
+      <c r="M34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -2239,12 +2235,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Flow sensor YF-S401 0.3-6 L/min</t>
+          <t>Mini submersible pump 3-9 V DC</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>5880 pulses per litre, JST-XH lead</t>
+          <t>for 5 V, about 0.2-0.3 A</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2260,16 +2256,16 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>AM Electronics</t>
+          <t>QuartzComponents</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>https://amelectronics.in/product/water-flow-sensor-yf-s401-flowmeter-0-3-6l-min-3-5mm-white/</t>
+          <t>https://quartzcomponents.com/products/3v-to-12v-mini-dc-submersible-pump</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>230</v>
+        <v>61</v>
       </c>
       <c r="K35" s="4">
         <f>ROUND(G35*J35,0)</f>
@@ -2280,7 +2276,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Rs 33 version out of stock; U-nozzle version Rs 61</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -2293,12 +2293,12 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Mini submersible pump 3-9 V DC</t>
+          <t>Enclosure REI IP-65-26 (TR top) 90x58x44</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>for 5 V, about 0.2-0.3 A</t>
+          <t>clear lid</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2314,16 +2314,16 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>QuartzComponents</t>
+          <t>REI Cabinets</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>https://quartzcomponents.com/products/3v-to-12v-mini-dc-submersible-pump</t>
+          <t>https://www.reicabinets.com/product?cid=16&amp;pid=479&amp;prodn=IP-65-26%20(TR%20Top)</t>
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>61</v>
+        <v>95</v>
       </c>
       <c r="K36" s="4">
         <f>ROUND(G36*J36,0)</f>
@@ -2334,11 +2334,7 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr">
-        <is>
-          <t>Rs 33 version out of stock; U-nozzle version Rs 61</t>
-        </is>
-      </c>
+      <c r="M36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -2351,37 +2347,37 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Enclosure REI IP-65-26 (TR top) 90x58x44</t>
+          <t>Nylon reverse-mount snap standoff 5 mm</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>clear lid</t>
+          <t>base taped to the box floor, head through the 4.2 mm PCB hole</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>H1-H3</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>REI Cabinets</t>
+          <t>Probots</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>https://www.reicabinets.com/product?cid=16&amp;pid=479&amp;prodn=IP-65-26%20(TR%20Top)</t>
+          <t>https://probots.co.in/5mm-nylon-reverse-mount-pcb-standoff-spacer.html</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="K37" s="4">
         <f>ROUND(G37*J37,0)</f>
@@ -2392,7 +2388,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>6 + 2 spare (Rs 10 below 25 pcs)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -2405,50 +2405,46 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Nylon reverse-mount snap standoff 5 mm</t>
+          <t>Double-sided foam tape (3M VHB type) squares</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>base taped to the box floor, head through the 4.2 mm PCB hole</t>
+          <t>about 10 x 10 mm, one per standoff</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>H1-H3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
         <v>6</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Probots</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>https://probots.co.in/5mm-nylon-reverse-mount-pcb-standoff-spacer.html</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr"/>
       <c r="J38" s="4" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="K38" s="4">
         <f>ROUND(G38*J38,0)</f>
         <v/>
       </c>
-      <c r="L38" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>6 + 2 spare (Rs 10 below 25 pcs)</t>
+          <t>One small roll</t>
         </is>
       </c>
     </row>
@@ -2463,12 +2459,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Double-sided foam tape (3M VHB type) squares</t>
+          <t>Cable gland PG7 nylon (3-6 mm cable)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>about 10 x 10 mm, one per standoff</t>
+          <t>USB, sensors, pump</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -2480,29 +2476,33 @@
         <v>6</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr"/>
+          <t>ElectroHeight</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>https://electroheight.com/PG7-cable-gland</t>
+        </is>
+      </c>
       <c r="J39" s="4" t="n">
-        <v>60</v>
+        <v>11.8</v>
       </c>
       <c r="K39" s="4">
         <f>ROUND(G39*J39,0)</f>
         <v/>
       </c>
-      <c r="L39" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
         </is>
       </c>
       <c r="M39" s="4" t="inlineStr">
         <is>
-          <t>One small roll</t>
+          <t>Single pieces (DNA Technology Rs 11.80)</t>
         </is>
       </c>
     </row>
@@ -2517,12 +2517,12 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Cable gland PG7 nylon (3-6 mm cable)</t>
+          <t>4-core cable 1 m (AHT20 stick)</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>USB, sensors, pump</t>
+          <t>e.g. 4 x 0.25 sq mm</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2531,36 +2531,32 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>ElectroHeight</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>https://electroheight.com/PG7-cable-gland</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="n">
-        <v>11.8</v>
+        <v>15</v>
       </c>
       <c r="K40" s="4">
         <f>ROUND(G40*J40,0)</f>
         <v/>
       </c>
-      <c r="L40" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
-          <t>Single pieces (DNA Technology Rs 11.80)</t>
+          <t>2 m</t>
         </is>
       </c>
     </row>
@@ -2575,12 +2571,12 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>4-core cable 1 m (AHT20 stick)</t>
+          <t>Silicone tube 1 m for the pump</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>e.g. 4 x 0.25 sq mm</t>
+          <t>match the pump outlet (about 7.5 mm OD)</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2601,7 +2597,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="K41" s="4">
         <f>ROUND(G41*J41,0)</f>
@@ -2619,69 +2615,35 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Kit items</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Silicone tube 1 m for the pump</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>match the pump outlet (about 7.5 mm OD)</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>Local market</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="K42" s="4">
-        <f>ROUND(G42*J42,0)</f>
-        <v/>
-      </c>
-      <c r="L42" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>2 m</t>
-        </is>
-      </c>
+      <c r="C42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
     </row>
     <row r="43">
-      <c r="C43" s="8" t="n"/>
-      <c r="K43" s="8" t="n"/>
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>LCSC order (SMD parts)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43">
+        <f>SUMIF(B6:B41,"SMD (JLC assembly or LCSC)",K6:K41)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>LCSC order (SMD parts)</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Indian suppliers / local</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2691,17 +2653,17 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
-      <c r="K44">
-        <f>SUMIF(B6:B42,"SMD (JLC assembly or LCSC)",K6:K42)</f>
+      <c r="K44" s="8">
+        <f>SUMIF(B6:B41,"Through-hole (India)",K6:K41)+SUMIF(B6:B41,"Kit items",K6:K41)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Indian suppliers / local</t>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL parts for 2 sample kits (+ LCSC shipping)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2711,28 +2673,8 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
-      <c r="K45" s="8">
-        <f>SUMIF(B6:B42,"Through-hole (India)",K6:K42)+SUMIF(B6:B42,"Kit items",K6:K42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL parts for 2 sample kits (+ LCSC shipping)</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" s="9">
-        <f>SUM(K6:K42)</f>
+      <c r="K45" s="9">
+        <f>SUM(K6:K41)</f>
         <v/>
       </c>
     </row>
@@ -2759,14 +2701,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2778,7 +2719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3205,21 +3146,21 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 red (PUMP)</t>
+          <t>LED 1206 yellow (PUMP, RELAY)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>YONGYUTAI YLED1206RFT, LCSC C37635751</t>
+          <t>YONGYUTAI YLED1206Y, LCSC C30584802</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D3, D7</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" s="4">
         <f>CEILING(F10*80,1)</f>
@@ -3232,11 +3173,11 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C37635751.html</t>
+          <t>https://www.lcsc.com/product-detail/C30584802.html</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K10" s="4">
         <f>ROUND(F10*J10,2)</f>
@@ -3268,17 +3209,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 yellow (FLOW)</t>
+          <t>LED 1206 red (STATUS)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>YLED1206Y, LCSC C30584802</t>
+          <t>YLED1206RFT, LCSC C37635751</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
@@ -3295,11 +3236,11 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C30584802.html</t>
+          <t>https://www.lcsc.com/product-detail/C37635751.html</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="K11" s="4">
         <f>ROUND(F11*J11,2)</f>
@@ -3327,17 +3268,17 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 green (STATUS)</t>
+          <t>LED 1206 yellow-green (FLOW)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>YLED1206GFT, LCSC C37635752</t>
+          <t>YLED1206YG 576 nm, LCSC C28310441</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
@@ -3354,11 +3295,11 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C37635752.html</t>
+          <t>https://www.lcsc.com/product-detail/C28310441.html</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="K12" s="4">
         <f>ROUND(F12*J12,2)</f>
@@ -3373,7 +3314,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Yellow-green (Vf ~2 V), not emerald green (Vf ~3 V): this LED runs from 3.3 V into the sensor output</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -3386,21 +3331,21 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>LED 1206 blue (RELAY)</t>
+          <t>Resistor 0805 1k</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>YLED1206B, LCSC C28310438</t>
+          <t>LCSC C17513</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>R3, R4, R12</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13" s="4">
         <f>CEILING(F13*80,1)</f>
@@ -3413,11 +3358,11 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C28310438.html</t>
+          <t>https://www.lcsc.com/product-detail/C17513.html</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>1.4</v>
+        <v>0.31</v>
       </c>
       <c r="K13" s="4">
         <f>ROUND(F13*J13,2)</f>
@@ -3432,11 +3377,7 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>Low stock at LCSC (450 on 2026-10-11)</t>
-        </is>
-      </c>
+      <c r="N13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -3449,21 +3390,21 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 1k</t>
+          <t>Resistor 0805 470R</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17513</t>
+          <t>LCSC C17710</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>R3, R4, R12</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4">
         <f>CEILING(F14*80,1)</f>
@@ -3476,11 +3417,11 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17513.html</t>
+          <t>https://www.lcsc.com/product-detail/C17710.html</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.31</v>
+        <v>0.43</v>
       </c>
       <c r="K14" s="4">
         <f>ROUND(F14*J14,2)</f>
@@ -3508,21 +3449,21 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 470R</t>
+          <t>Resistor 0805 10k</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17710</t>
+          <t>LCSC C17414</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R6, R7</t>
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G15" s="4">
         <f>CEILING(F15*80,1)</f>
@@ -3535,11 +3476,11 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17710.html</t>
+          <t>https://www.lcsc.com/product-detail/C17414.html</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.43</v>
+        <v>0.3</v>
       </c>
       <c r="K15" s="4">
         <f>ROUND(F15*J15,2)</f>
@@ -3567,17 +3508,17 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 10k</t>
+          <t>Resistor 0805 4.7k</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17414</t>
+          <t>LCSC C17673</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>R6, R7</t>
+          <t>R8, R9</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
@@ -3594,11 +3535,11 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17414.html</t>
+          <t>https://www.lcsc.com/product-detail/C17673.html</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="K16" s="4">
         <f>ROUND(F16*J16,2)</f>
@@ -3626,21 +3567,21 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Resistor 0805 4.7k</t>
+          <t>Capacitor 0805 100nF 50V</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>LCSC C17673</t>
+          <t>LCSC C49678</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>R8, R9</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" s="4">
         <f>CEILING(F17*80,1)</f>
@@ -3653,11 +3594,11 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C17673.html</t>
+          <t>https://www.lcsc.com/product-detail/C49678.html</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.45</v>
+        <v>1.2</v>
       </c>
       <c r="K17" s="4">
         <f>ROUND(F17*J17,2)</f>
@@ -3685,17 +3626,17 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Capacitor 0805 100nF 50V</t>
+          <t>Capacitor 0805 10uF 25V (on the stick)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>LCSC C49678</t>
+          <t>LCSC C15850</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C1 (stick)</t>
         </is>
       </c>
       <c r="F18" s="4" t="n">
@@ -3712,11 +3653,11 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C49678.html</t>
+          <t>https://www.lcsc.com/product-detail/C15850.html</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>1.2</v>
+        <v>4.5</v>
       </c>
       <c r="K18" s="4">
         <f>ROUND(F18*J18,2)</f>
@@ -3744,17 +3685,17 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Capacitor 0805 10uF 25V (on the stick)</t>
+          <t>JLC SMT assembly share (if JLC assembles)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>LCSC C15850</t>
+          <t>setup + stencil + 3 extended-part fees (DS1307, AHT20, ULN2003A) over 80 sets</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>C1 (stick)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F19" s="4" t="n">
@@ -3766,16 +3707,16 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>LCSC</t>
+          <t>JLCPCB / WhyPCB</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>https://www.lcsc.com/product-detail/C15850.html</t>
+          <t>https://jlcpcb.com/smt-assembly</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>4.5</v>
+        <v>25</v>
       </c>
       <c r="K19" s="4">
         <f>ROUND(F19*J19,2)</f>
@@ -3785,12 +3726,16 @@
         <f>ROUND(F19*80*J19,0)</f>
         <v/>
       </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Skip if hand-assembled; the AHT20 still needs reflow or hot air</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -3798,22 +3743,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>SMD (JLC assembly or LCSC)</t>
+          <t>Through-hole (India)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>JLC SMT assembly share (if JLC assembles)</t>
+          <t>ESP32-C3 Super Mini USB-C</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>setup + stencil + 3 extended-part fees (DS1307, AHT20, ULN2003A) over 80 sets</t>
+          <t>plugs into the two 1x8 sockets</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="F20" s="4" t="n">
@@ -3825,16 +3770,16 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>JLCPCB / WhyPCB</t>
+          <t>Robosap</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>https://jlcpcb.com/smt-assembly</t>
+          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>25</v>
+        <v>238.36</v>
       </c>
       <c r="K20" s="4">
         <f>ROUND(F20*J20,2)</f>
@@ -3844,14 +3789,14 @@
         <f>ROUND(F20*80*J20,0)</f>
         <v/>
       </c>
-      <c r="M20" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>Skip if hand-assembled; the AHT20 still needs reflow or hot air</t>
+          <t>Rs 202 + GST; check the pin order against the 1:1 print</t>
         </is>
       </c>
     </row>
@@ -3866,12 +3811,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>ESP32-C3 Super Mini USB-C</t>
+          <t>Female header 1x8 2.54 mm</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>plugs into the two 1x8 sockets</t>
+          <t>Super Mini socket, 8.5 mm tall</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -3880,7 +3825,7 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="4">
         <f>CEILING(F21*80,1)</f>
@@ -3888,16 +3833,16 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Robosap</t>
+          <t>Sharvi Electronics</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>https://robosap.in/product/esp32-c3-super-mini-usb-c-type-development-board/</t>
+          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>238.36</v>
+        <v>10.72</v>
       </c>
       <c r="K21" s="4">
         <f>ROUND(F21*J21,2)</f>
@@ -3912,11 +3857,7 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t>Rs 202 + GST; check the pin order against the 1:1 print</t>
-        </is>
-      </c>
+      <c r="N21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -3929,21 +3870,21 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Female header 1x8 2.54 mm</t>
+          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Super Mini socket, 8.5 mm tall</t>
+          <t>SPST-NO, sealed, VDE reinforced</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4">
         <f>CEILING(F22*80,1)</f>
@@ -3951,16 +3892,16 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Sharvi Electronics</t>
+          <t>techiesms</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>https://sharvielectronics.com/product/8x1-8pin-female-berg-strip-break-away-header-straight-2-54mm-pitch/</t>
+          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>10.72</v>
+        <v>42</v>
       </c>
       <c r="K22" s="4">
         <f>ROUND(F22*J22,2)</f>
@@ -3975,7 +3916,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>Rs 210 for a pack of 5</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -3988,17 +3933,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Relay Hongfa HF46F 5 V, 5 A 250 VAC</t>
+          <t>CR2032 with 3 solder tabs, vertical</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>SPST-NO, sealed, VDE reinforced</t>
+          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>BT1</t>
         </is>
       </c>
       <c r="F23" s="4" t="n">
@@ -4010,16 +3955,16 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>techiesms</t>
+          <t>Rajiv Electronics</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>https://techiesms.com/product/hf46f-5v-pcb-sealed-relaypack-of-5/</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>42</v>
+        <v>29.5</v>
       </c>
       <c r="K23" s="4">
         <f>ROUND(F23*J23,2)</f>
@@ -4036,7 +3981,7 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Rs 210 for a pack of 5</t>
+          <t>Measure the - leg offset on the first lot (footprint assumes 4.0 mm)</t>
         </is>
       </c>
     </row>
@@ -4051,21 +3996,21 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>CR2032 with 3 solder tabs, vertical</t>
+          <t>ALTERNATIVE: CR2032 holder (vertical, 3 pins, Rajiv RBH-2) + loose CR2032 cell</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2 x + legs 15.2 mm apart, 1 x - leg</t>
+          <t>3-pin vertical holder; pin positions to be measured against the tabbed-cell pads</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>BT1</t>
+          <t>BT1 (alt)</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="4">
         <f>CEILING(F24*80,1)</f>
@@ -4078,11 +4023,11 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>https://rajivelectronics.com/product/cr2032-3v-lithium-battery-vertical-3-pin-pc-mount-battery</t>
+          <t>https://rajivelectronics.com/product/cr2032-3v-pcb-mount-vertical-battery-holder</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>29.5</v>
+        <v>11.8</v>
       </c>
       <c r="K24" s="4">
         <f>ROUND(F24*J24,2)</f>
@@ -4099,7 +4044,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Measure the - leg offset on the first lot (footprint assumes 4.0 mm)</t>
+          <t>Rs 11.80 + a loose CR2032 (about Rs 20). Replaceable cell. Measure a sample: if its 3 pins match the tabbed-cell pads it drops in, otherwise we add its pads</t>
         </is>
       </c>
     </row>
@@ -4114,21 +4059,21 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>ALTERNATIVE: CR2032 holder (vertical, 3 pins, Rajiv RBH-2) + loose CR2032 cell</t>
+          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>3-pin vertical holder; pin positions to be measured against the tabbed-cell pads</t>
+          <t>cylindrical</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>BT1 (alt)</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="4">
         <f>CEILING(F25*80,1)</f>
@@ -4136,16 +4081,16 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Rajiv Electronics</t>
+          <t>Magno Teknik</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>https://rajivelectronics.com/product/cr2032-3v-pcb-mount-vertical-battery-holder</t>
+          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>11.8</v>
+        <v>14</v>
       </c>
       <c r="K25" s="4">
         <f>ROUND(F25*J25,2)</f>
@@ -4162,7 +4107,7 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>Rs 11.80 + a loose CR2032 (about Rs 20). Replaceable cell. Measure a sample: if its 3 pins match the tabbed-cell pads it drops in, otherwise we add its pads</t>
+          <t>Rs 14 at 100+; local market about Rs 4-8</t>
         </is>
       </c>
     </row>
@@ -4177,17 +4122,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Crystal 32.768 kHz 2x6 mm, 12.5 pF</t>
+          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>cylindrical</t>
+          <t>radial 5 x 11</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
@@ -4199,16 +4144,12 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Magno Teknik</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>https://store.magnoteknik.com/product/mtcr2632r768k/</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" s="4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="K26" s="4">
         <f>ROUND(F26*J26,2)</f>
@@ -4218,16 +4159,12 @@
         <f>ROUND(F26*80*J26,0)</f>
         <v/>
       </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t>Rs 14 at 100+; local market about Rs 4-8</t>
-        </is>
-      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -4240,17 +4177,17 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Electrolytic 220 uF 10 V, 5 mm dia, 2.0 mm pitch</t>
+          <t>Screw terminal 3.5 mm 2P (PUMP)</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>radial 5 x 11</t>
+          <t>KF350-2P / DG350 (Phoenix PT-1,5 footprint), horizontal</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
@@ -4262,12 +4199,12 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
+          <t>Local market (Lamington Rd / SP Road)</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr"/>
       <c r="J27" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K27" s="4">
         <f>ROUND(F27*J27,2)</f>
@@ -4282,7 +4219,11 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>3.5 mm pitch blocks interlock: buy 2P and 3P and join them</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -4295,17 +4236,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.5 mm 2P (PUMP)</t>
+          <t>Screw terminal 3.5 mm 4P (I2C)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>KF350-2P / DG350 (Phoenix PT-1,5 footprint), horizontal</t>
+          <t>KF350 2P + 2P joined</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
@@ -4317,12 +4258,12 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Local market (Lamington Rd / SP Road)</t>
+          <t>Local market</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr"/>
       <c r="J28" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K28" s="4">
         <f>ROUND(F28*J28,2)</f>
@@ -4339,7 +4280,7 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>3.5 mm pitch blocks interlock: buy 2P and 3P and join them</t>
+          <t>Wire entry faces the board edge</t>
         </is>
       </c>
     </row>
@@ -4354,17 +4295,17 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.5 mm 4P (I2C)</t>
+          <t>Screw terminal 3.5 mm 5P (AUX)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>KF350 2P + 2P joined</t>
+          <t>KF350 2P + 3P joined</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="F29" s="4" t="n">
@@ -4381,7 +4322,7 @@
       </c>
       <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K29" s="4">
         <f>ROUND(F29*J29,2)</f>
@@ -4396,11 +4337,7 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>Wire entry faces the board edge</t>
-        </is>
-      </c>
+      <c r="N29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -4413,21 +4350,21 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.5 mm 5P (AUX)</t>
+          <t>Screw terminal 3.5 mm 3P (FLOW, field builds)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>KF350 2P + 3P joined</t>
+          <t>KF350-3P; fits the same holes as the JST-XH</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J4 (alt)</t>
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" s="4">
         <f>CEILING(F30*80,1)</f>
@@ -4440,7 +4377,7 @@
       </c>
       <c r="I30" s="4" t="inlineStr"/>
       <c r="J30" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K30" s="4">
         <f>ROUND(F30*J30,2)</f>
@@ -4455,7 +4392,11 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>FG1 / long cable: fit this instead of the JST-XH header</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -4468,21 +4409,21 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Screw terminal 3.5 mm 3P (FLOW, field builds)</t>
+          <t>Pluggable header 5.08 mm 2P, vertical, + plug (RELAY 230 V)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>KF350-3P; fits the same holes as the JST-XH</t>
+          <t>MSTBVA 2,5/2-G-5,08 type (2EDG-V 5.08) with 2EDGK plug</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>J4 (alt)</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" s="4">
         <f>CEILING(F31*80,1)</f>
@@ -4493,9 +4434,13 @@
           <t>Local market</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>https://www.electronicscomp.com/kf301-2-pin-5.08mm-pitch-plug-in-screw-terminal-block-connector</t>
+        </is>
+      </c>
       <c r="J31" s="4" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K31" s="4">
         <f>ROUND(F31*J31,2)</f>
@@ -4512,7 +4457,7 @@
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>FG1 / long cable: fit this instead of the JST-XH header</t>
+          <t>Same pluggable family as FG1's relay connector; buy header and plug as a pair (link: similar plug-in block)</t>
         </is>
       </c>
     </row>
@@ -4527,17 +4472,17 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Pluggable header 5.08 mm 2P, vertical, + plug (RELAY 230 V)</t>
+          <t>JST-XH 3-pin male header, straight 2.5 mm (FLOW, student builds)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>MSTBVA 2,5/2-G-5,08 type (2EDG-V 5.08) with 2EDGK plug</t>
+          <t>B3B-XH-A type; shares the footprint with the 3.5 mm terminal</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
@@ -4549,16 +4494,16 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
+          <t>DNA Technology</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>https://www.electronicscomp.com/kf301-2-pin-5.08mm-pitch-plug-in-screw-terminal-block-connector</t>
+          <t>https://www.dnatechindia.com/3-pin-2-50mm-jst-xh-straight-male-connector-buy-in-india.html</t>
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>15</v>
+        <v>4.56</v>
       </c>
       <c r="K32" s="4">
         <f>ROUND(F32*J32,2)</f>
@@ -4568,14 +4513,14 @@
         <f>ROUND(F32*80*J32,0)</f>
         <v/>
       </c>
-      <c r="M32" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
         </is>
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Same pluggable family as FG1's relay connector; buy header and plug as a pair (link: similar plug-in block)</t>
+          <t>Mates with the YF-S401 plug</t>
         </is>
       </c>
     </row>
@@ -4590,21 +4535,21 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>JST-XH 3-pin male header, straight 2.5 mm (FLOW, student builds)</t>
+          <t>Pin header 1x4 2.54 mm (AHT20 stick cable end, optional)</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>B3B-XH-A type; shares the footprint with the 3.5 mm terminal</t>
+          <t>or solder the cable directly</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J1 (stick)</t>
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" s="4">
         <f>CEILING(F33*80,1)</f>
@@ -4612,16 +4557,12 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>DNA Technology</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>https://www.dnatechindia.com/3-pin-2-50mm-jst-xh-straight-male-connector-buy-in-india.html</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
       <c r="J33" s="4" t="n">
-        <v>4.56</v>
+        <v>1</v>
       </c>
       <c r="K33" s="4">
         <f>ROUND(F33*J33,2)</f>
@@ -4631,14 +4572,14 @@
         <f>ROUND(F33*80*J33,0)</f>
         <v/>
       </c>
-      <c r="M33" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
-          <t>Mates with the YF-S401 plug</t>
+          <t>Not needed if the cable is soldered</t>
         </is>
       </c>
     </row>
@@ -4648,26 +4589,26 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Through-hole (India)</t>
+          <t>Kit items</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Pin header 1x4 2.54 mm (AHT20 stick cable end, optional)</t>
+          <t>Flow sensor YF-S401 0.3-6 L/min</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>or solder the cable directly</t>
+          <t>5880 pulses per litre, JST-XH lead</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>J1 (stick)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="4">
         <f>CEILING(F34*80,1)</f>
@@ -4675,12 +4616,16 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr"/>
+          <t>AM Electronics</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>https://amelectronics.in/product/water-flow-sensor-yf-s401-flowmeter-0-3-6l-min-3-5mm-white/</t>
+        </is>
+      </c>
       <c r="J34" s="4" t="n">
-        <v>1</v>
+        <v>230</v>
       </c>
       <c r="K34" s="4">
         <f>ROUND(F34*J34,2)</f>
@@ -4690,14 +4635,14 @@
         <f>ROUND(F34*80*J34,0)</f>
         <v/>
       </c>
-      <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
         </is>
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>Not needed if the cable is soldered</t>
+          <t>Check the plug order: GND, 5V, SIG</t>
         </is>
       </c>
     </row>
@@ -4712,12 +4657,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Flow sensor YF-S401 0.3-6 L/min</t>
+          <t>Mini submersible pump 3-9 V DC</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>5880 pulses per litre, JST-XH lead</t>
+          <t>for 5 V, about 0.2-0.3 A</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -4734,16 +4679,16 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>AM Electronics</t>
+          <t>QuartzComponents</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>https://amelectronics.in/product/water-flow-sensor-yf-s401-flowmeter-0-3-6l-min-3-5mm-white/</t>
+          <t>https://quartzcomponents.com/products/3v-to-12v-mini-dc-submersible-pump</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>230</v>
+        <v>33</v>
       </c>
       <c r="K35" s="4">
         <f>ROUND(F35*J35,2)</f>
@@ -4760,7 +4705,7 @@
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>Check the plug order: GND, 5V, SIG</t>
+          <t>Out of stock on 2026-10-10; U-nozzle version Rs 61: quartzcomponents.com/collections/dc-motors/products/3v-to-9v-mini-dc-submersible-pump-u-type-nozzel</t>
         </is>
       </c>
     </row>
@@ -4775,12 +4720,12 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Mini submersible pump 3-9 V DC</t>
+          <t>Enclosure REI IP-65-26 (TR top) 90x58x44</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>for 5 V, about 0.2-0.3 A</t>
+          <t>clear lid</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -4797,16 +4742,16 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>QuartzComponents</t>
+          <t>REI Cabinets</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>https://quartzcomponents.com/products/3v-to-12v-mini-dc-submersible-pump</t>
+          <t>https://www.reicabinets.com/product?cid=16&amp;pid=479&amp;prodn=IP-65-26%20(TR%20Top)</t>
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="K36" s="4">
         <f>ROUND(F36*J36,2)</f>
@@ -4821,11 +4766,7 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t>Out of stock on 2026-10-10; U-nozzle version Rs 61: quartzcomponents.com/collections/dc-motors/products/3v-to-9v-mini-dc-submersible-pump-u-type-nozzel</t>
-        </is>
-      </c>
+      <c r="N36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -4838,21 +4779,21 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Enclosure REI IP-65-26 (TR top) 90x58x44</t>
+          <t>Nylon reverse-mount snap standoff 5 mm</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>clear lid</t>
+          <t>base taped to the box floor, head through the 4.2 mm PCB hole</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>H1-H3</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G37" s="4">
         <f>CEILING(F37*80,1)</f>
@@ -4860,16 +4801,16 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>REI Cabinets</t>
+          <t>Probots</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>https://www.reicabinets.com/product?cid=16&amp;pid=479&amp;prodn=IP-65-26%20(TR%20Top)</t>
+          <t>https://probots.co.in/5mm-nylon-reverse-mount-pcb-standoff-spacer.html</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>95</v>
+        <v>9.4</v>
       </c>
       <c r="K37" s="4">
         <f>ROUND(F37*J37,2)</f>
@@ -4884,7 +4825,11 @@
           <t>quoted</t>
         </is>
       </c>
-      <c r="N37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Rs 9.40 at 50+, Rs 8.50 at 100+</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -4897,17 +4842,17 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Nylon reverse-mount snap standoff 5 mm</t>
+          <t>Double-sided foam tape (3M VHB type) squares</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>base taped to the box floor, head through the 4.2 mm PCB hole</t>
+          <t>about 10 x 10 mm, one per standoff</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>H1-H3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F38" s="4" t="n">
@@ -4919,16 +4864,12 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Probots</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>https://probots.co.in/5mm-nylon-reverse-mount-pcb-standoff-spacer.html</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr"/>
       <c r="J38" s="4" t="n">
-        <v>9.4</v>
+        <v>1</v>
       </c>
       <c r="K38" s="4">
         <f>ROUND(F38*J38,2)</f>
@@ -4938,16 +4879,12 @@
         <f>ROUND(F38*80*J38,0)</f>
         <v/>
       </c>
-      <c r="M38" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="N38" s="4" t="inlineStr">
-        <is>
-          <t>Rs 9.40 at 50+, Rs 8.50 at 100+</t>
-        </is>
-      </c>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -4960,12 +4897,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Double-sided foam tape (3M VHB type) squares</t>
+          <t>Cable gland PG7 nylon (3-6 mm cable)</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>about 10 x 10 mm, one per standoff</t>
+          <t>USB, sensors, pump</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -4982,12 +4919,16 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Local market</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr"/>
+          <t>ElectroHeight</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>https://electroheight.com/PG7-cable-gland</t>
+        </is>
+      </c>
       <c r="J39" s="4" t="n">
-        <v>1</v>
+        <v>2.05</v>
       </c>
       <c r="K39" s="4">
         <f>ROUND(F39*J39,2)</f>
@@ -4997,12 +4938,16 @@
         <f>ROUND(F39*80*J39,0)</f>
         <v/>
       </c>
-      <c r="M39" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="N39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>quoted</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Rs 205 per 100; single pieces about Rs 12 (dnatechindia.com/pg7-cable-gland-buy-in-india.html)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -5015,12 +4960,12 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Cable gland PG7 nylon (3-6 mm cable)</t>
+          <t>4-core cable 1 m (AHT20 stick)</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>USB, sensors, pump</t>
+          <t>e.g. 4 x 0.25 sq mm</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -5029,7 +4974,7 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G40" s="4">
         <f>CEILING(F40*80,1)</f>
@@ -5037,16 +4982,12 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>ElectroHeight</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>https://electroheight.com/PG7-cable-gland</t>
-        </is>
-      </c>
+          <t>Local market</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="n">
-        <v>2.05</v>
+        <v>15</v>
       </c>
       <c r="K40" s="4">
         <f>ROUND(F40*J40,2)</f>
@@ -5056,16 +4997,12 @@
         <f>ROUND(F40*80*J40,0)</f>
         <v/>
       </c>
-      <c r="M40" s="4" t="inlineStr">
-        <is>
-          <t>quoted</t>
-        </is>
-      </c>
-      <c r="N40" s="4" t="inlineStr">
-        <is>
-          <t>Rs 205 per 100; single pieces about Rs 12 (dnatechindia.com/pg7-cable-gland-buy-in-india.html)</t>
-        </is>
-      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -5078,12 +5015,12 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>4-core cable 1 m (AHT20 stick)</t>
+          <t>Silicone tube 1 m for the pump</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>e.g. 4 x 0.25 sq mm</t>
+          <t>match the pump outlet (about 7.5 mm OD)</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -5105,7 +5042,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="K41" s="4">
         <f>ROUND(F41*J41,2)</f>
@@ -5123,71 +5060,40 @@
       <c r="N41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Kit items</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Silicone tube 1 m for the pump</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>match the pump outlet (about 7.5 mm OD)</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="4">
-        <f>CEILING(F42*80,1)</f>
-        <v/>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>Local market</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="K42" s="4">
-        <f>ROUND(F42*J42,2)</f>
-        <v/>
-      </c>
-      <c r="L42" s="4">
-        <f>ROUND(F42*80*J42,0)</f>
-        <v/>
-      </c>
-      <c r="M42" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="N42" s="4" t="inlineStr"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
+      <c r="L42" s="8" t="n"/>
     </row>
     <row r="43">
-      <c r="C43" s="8" t="n"/>
-      <c r="K43" s="8" t="n"/>
-      <c r="L43" s="8" t="n"/>
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Subtotal PCB + board parts</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43">
+        <f>SUMIF(B5:B41,"PCB",K5:K41)+SUMIF(B5:B41,"SMD (JLC assembly or LCSC)",K5:K41)+SUMIF(B5:B41,"Through-hole (India)",K5:K41)</f>
+        <v/>
+      </c>
+      <c r="L43">
+        <f>SUMIF(B5:B41,"PCB",L5:L41)+SUMIF(B5:B41,"SMD (JLC assembly or LCSC)",L5:L41)+SUMIF(B5:B41,"Through-hole (India)",L5:L41)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Subtotal PCB + board parts</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Subtotal kit items</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -5197,21 +5103,21 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
-      <c r="K44">
-        <f>SUMIF(B5:B42,"PCB",K5:K42)+SUMIF(B5:B42,"SMD (JLC assembly or LCSC)",K5:K42)+SUMIF(B5:B42,"Through-hole (India)",K5:K42)</f>
-        <v/>
-      </c>
-      <c r="L44">
-        <f>SUMIF(B5:B42,"PCB",L5:L42)+SUMIF(B5:B42,"SMD (JLC assembly or LCSC)",L5:L42)+SUMIF(B5:B42,"Through-hole (India)",L5:L42)</f>
+      <c r="K44" s="8">
+        <f>SUMIF(B5:B41,"Kit items",K5:K41)</f>
+        <v/>
+      </c>
+      <c r="L44" s="8">
+        <f>SUMIF(B5:B41,"Kit items",L5:L41)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Subtotal kit items</t>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL per kit / per batch</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -5221,36 +5127,12 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
-      <c r="K45" s="8">
-        <f>SUMIF(B5:B42,"Kit items",K5:K42)</f>
-        <v/>
-      </c>
-      <c r="L45" s="8">
-        <f>SUMIF(B5:B42,"Kit items",L5:L42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL per kit / per batch</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" s="9">
-        <f>SUM(K5:K42)</f>
-        <v/>
-      </c>
-      <c r="L46" s="9">
-        <f>SUM(L5:L42)</f>
+      <c r="K45" s="9">
+        <f>SUM(K5:K41)</f>
+        <v/>
+      </c>
+      <c r="L45" s="9">
+        <f>SUM(L5:L41)</f>
         <v/>
       </c>
     </row>
@@ -5277,14 +5159,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ASC Mini-C3 panel: plain tabs (no mouse bites); 10 panels ordered
- Mouse-bite holes removed: WhyPCB says JLC may not accept them
  (MOUSE_BITES flag in tools/panel.py keeps the option). Plain tabs,
  narrowed to ~2 mm at the panel edges and ~5 mm at the slot crossings.
  Panel DRC: 0 errors.
- PANEL-README, README, BOM wording: routed slots, plain tabs, no V-cut,
  no mouse bites.
- Sourcing: 10 panels (40 Minis + 20 sticks) ordered from WhyPCB for
  Rs 2,000 on 2026-10-14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products/ASC-StudentKit/hardware/MiniC3/sourcing/ASC-MiniC3-sourcing-BOM.xlsx
+++ b/products/ASC-StudentKit/hardware/MiniC3/sourcing/ASC-MiniC3-sourcing-BOM.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>98 x 98 panel = 4 Minis + 2 sticks, 2 layers, 1.6 mm, HASL; 2 mm routed slots + mouse bites (no V-cut)</t>
+          <t>98 x 98 panel = 4 Minis + 2 sticks, 2 layers, 1.6 mm, HASL; 2 mm routed slots + plain tabs (no V-cut, no mouse bites)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -602,7 +602,7 @@
         <v>0.5</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="J6" s="3" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="K6" s="3">
         <f>ROUND(G6*J6,0)</f>
@@ -628,7 +628,7 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>5 panels = 20 Minis + 10 sticks; WhyPCB Rs 1,500 total (slots + mouse bites, no V-cut)</t>
+          <t>ORDERED 2026-10-14: 10 panels = 40 Minis + 20 sticks, WhyPCB Rs 2,000 total (routed slots + plain tabs)</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>98 x 98 panel = 4 Minis + 2 sticks, 2 layers, 1.6 mm, HASL; 2 mm routed slots + mouse bites (no V-cut)</t>
+          <t>98 x 98 panel = 4 Minis + 2 sticks, 2 layers, 1.6 mm, HASL; 2 mm routed slots + plain tabs (no V-cut, no mouse bites)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">

</xml_diff>